<commit_message>
Ver6 - 12 months display corrected
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_FU_PHONE/Forms/MADTRIAL_FU_PHONE/MADTRIAL_FU_PHONE.xlsx
+++ b/app/config/tables/MADTRIAL_FU_PHONE/Forms/MADTRIAL_FU_PHONE/MADTRIAL_FU_PHONE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_FU_PHONE\Forms\MADTRIAL_FU_PHONE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MAD\ver6\MADtrial\app\config\tables\MADTRIAL_FU_PHONE\Forms\MADTRIAL_FU_PHONE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B6D433-15AB-4D90-A8D3-DC3640758797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F83A7C-F559-4520-B8A5-717AB13FDF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="412">
   <si>
     <t>setting_name</t>
   </si>
@@ -1290,6 +1290,9 @@
   </si>
   <si>
     <t>Sarampo2</t>
+  </si>
+  <si>
+    <t>Makci</t>
   </si>
 </sst>
 </file>
@@ -1735,7 +1738,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>20250725</v>
+        <v>20260731</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -5490,7 +5493,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.54296875" bestFit="1" customWidth="1"/>
@@ -5734,7 +5737,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>57</v>
       </c>
@@ -5748,7 +5751,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>57</v>
       </c>
@@ -5762,7 +5765,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>57</v>
       </c>
@@ -5776,7 +5779,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -5790,7 +5793,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -5807,7 +5810,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -5821,7 +5824,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>57</v>
       </c>
@@ -5835,7 +5838,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>51</v>
       </c>
@@ -5850,7 +5853,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>51</v>
       </c>
@@ -5865,57 +5868,67 @@
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="E26" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E27" t="s">
         <v>98</v>
       </c>
-      <c r="B27" t="str">
+      <c r="F27" t="str">
         <f>"2"</f>
         <v>2</v>
       </c>
-      <c r="C27" t="s">
+      <c r="G27" t="s">
         <v>400</v>
       </c>
-      <c r="D27" t="s">
+      <c r="H27" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E28" t="s">
         <v>98</v>
       </c>
-      <c r="B28" t="str">
+      <c r="F28" t="str">
         <f>"3"</f>
         <v>3</v>
       </c>
-      <c r="C28" t="s">
+      <c r="G28" t="s">
         <v>398</v>
       </c>
-      <c r="D28" t="s">
+      <c r="H28" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>98</v>
       </c>
       <c r="B29" t="str">
+        <f>"14"</f>
+        <v>14</v>
+      </c>
+      <c r="C29" t="s">
+        <v>411</v>
+      </c>
+      <c r="D29" t="s">
+        <v>411</v>
+      </c>
+      <c r="E29" t="str">
         <f>"10"</f>
         <v>10</v>
       </c>
-      <c r="C29" t="s">
+      <c r="F29" t="s">
         <v>397</v>
       </c>
-      <c r="D29" t="s">
+      <c r="G29" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -5933,7 +5946,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>98</v>
       </c>
@@ -5948,7 +5961,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>98</v>
       </c>

</xml_diff>